<commit_message>
CAR Mujeres: codo PVC 4" x 45 en el RESUMEN (1.4.4.5.3.2), numeracion de accesorios igual a la PLANILLA
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_mujeres/METRADO_DRENAJE_PLUVIAL_CAR_MUJERES_09-10-2026_CON_BANCAS.xlsx
+++ b/entregables_mujeres/METRADO_DRENAJE_PLUVIAL_CAR_MUJERES_09-10-2026_CON_BANCAS.xlsx
@@ -37,7 +37,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'METRADO CANALETAS'!$A$1:$L$53</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'METRADO MONTANTES'!$A$1:$R$69</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'PLANILLA GENERAL DE METRADOS'!$A$1:$L$326</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">RESUMEN!$A$1:$D$84</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">RESUMEN!$A$1:$D$85</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'CONCRETO EN CUNETAS'!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'ENCOFRADO Y DESENCOFRADO'!$2:$7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'METRADO CANALETAS'!$1:$10</definedName>
@@ -4911,7 +4911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.08984375" style="4" customWidth="1"/>
@@ -5562,14 +5562,14 @@
         <v>99</v>
       </c>
       <c r="B50" s="13" t="s">
-        <v>100</v>
+        <v>641</v>
       </c>
       <c r="C50" s="15" t="s">
         <v>60</v>
       </c>
       <c r="D50" s="16" t="n">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K162</f>
-        <v>106.0</v>
+        <f aca="false">+'PLANILLA GENERAL DE METRADOS'!K161</f>
+        <v>2.0</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.35">
@@ -5577,462 +5577,477 @@
         <v>101</v>
       </c>
       <c r="B51" s="13" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C51" s="15" t="s">
         <v>60</v>
       </c>
       <c r="D51" s="16" t="n">
+        <f>+'PLANILLA GENERAL DE METRADOS'!K162</f>
+        <v>106.0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A52" s="13" t="s">
+        <v>640</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C52" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="D52" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K163</f>
         <v>90.0</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A52" s="13" t="s">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A53" s="13" t="s">
         <v>658</v>
       </c>
-      <c r="B52" s="19" t="s">
+      <c r="B53" s="19" t="s">
         <v>659</v>
       </c>
-      <c r="C52" s="15"/>
-      <c r="D52" s="16"/>
-    </row>
-    <row r="53" spans="1:4" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="202" t="s">
+      <c r="C53" s="15"/>
+      <c r="D53" s="16"/>
+    </row>
+    <row r="54" spans="1:4" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="202" t="s">
         <v>660</v>
       </c>
-      <c r="B53" s="203" t="s">
+      <c r="B54" s="203" t="s">
         <v>661</v>
       </c>
-      <c r="C53" s="204" t="s">
+      <c r="C54" s="204" t="s">
         <v>57</v>
       </c>
-      <c r="D53" s="205" t="n">
+      <c r="D54" s="205" t="n">
         <f aca="false">+'PLANILLA GENERAL DE METRADOS'!K166</f>
         <v>32.0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="202" t="s">
+    <row r="55" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="202" t="s">
         <v>662</v>
       </c>
-      <c r="B54" s="203" t="s">
+      <c r="B55" s="203" t="s">
         <v>663</v>
       </c>
-      <c r="C54" s="204" t="s">
+      <c r="C55" s="204" t="s">
         <v>60</v>
       </c>
-      <c r="D54" s="205" t="n">
+      <c r="D55" s="205" t="n">
         <f aca="false">+'PLANILLA GENERAL DE METRADOS'!K167</f>
         <v>32.0</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="202" t="s">
+    <row r="56" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="202" t="s">
         <v>664</v>
       </c>
-      <c r="B55" s="203" t="s">
+      <c r="B56" s="203" t="s">
         <v>80</v>
       </c>
-      <c r="C55" s="204" t="s">
+      <c r="C56" s="204" t="s">
         <v>60</v>
       </c>
-      <c r="D55" s="205" t="n">
+      <c r="D56" s="205" t="n">
         <f aca="false">+'PLANILLA GENERAL DE METRADOS'!K168</f>
         <v>32.0</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="202" t="s">
+    <row r="57" spans="1:4" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="202" t="s">
         <v>665</v>
       </c>
-      <c r="B56" s="203" t="s">
+      <c r="B57" s="203" t="s">
         <v>666</v>
       </c>
-      <c r="C56" s="204" t="s">
+      <c r="C57" s="204" t="s">
         <v>60</v>
       </c>
-      <c r="D56" s="205" t="n">
+      <c r="D57" s="205" t="n">
         <f aca="false">+'PLANILLA GENERAL DE METRADOS'!K169</f>
         <v>16.0</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A57" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="B57" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C57" s="12"/>
-      <c r="D57" s="12"/>
-    </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>15</v>
+        <v>104</v>
       </c>
       <c r="C58" s="12"/>
       <c r="D58" s="12"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A59" s="13" t="s">
+      <c r="A59" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B59" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C59" s="12"/>
+      <c r="D59" s="12"/>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A60" s="13" t="s">
         <v>106</v>
       </c>
-      <c r="B59" s="14" t="s">
+      <c r="B60" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="C59" s="15" t="s">
+      <c r="C60" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D59" s="16" t="n">
+      <c r="D60" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K173</f>
         <v>255.361098</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A60" s="13" t="s">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A61" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="B60" s="14" t="s">
+      <c r="B61" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="C60" s="15" t="s">
+      <c r="C61" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D60" s="16" t="n">
+      <c r="D61" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K184</f>
         <v>255.361098</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A61" s="12" t="s">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A62" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="B61" s="12" t="s">
+      <c r="B62" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C61" s="12"/>
-      <c r="D61" s="12"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A62" s="13" t="s">
+      <c r="C62" s="12"/>
+      <c r="D62" s="12"/>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A63" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="B62" s="14" t="s">
+      <c r="B63" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="C62" s="15" t="s">
+      <c r="C63" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D62" s="16" t="n">
+      <c r="D63" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K196</f>
         <v>180.6554745</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A63" s="13" t="s">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A64" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="B63" s="14" t="s">
+      <c r="B64" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="C63" s="15" t="s">
+      <c r="C64" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D63" s="16" t="n">
+      <c r="D64" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K207</f>
         <v>239.4967</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A64" s="13" t="s">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A65" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="B64" s="14" t="s">
+      <c r="B65" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C64" s="15" t="s">
+      <c r="C65" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D64" s="16" t="n">
+      <c r="D65" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K219</f>
         <v>10.2</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A65" s="13" t="s">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A66" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="B65" s="14" t="s">
+      <c r="B66" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C65" s="15" t="s">
+      <c r="C66" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D65" s="16" t="n">
+      <c r="D66" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K231</f>
         <v>213.069343125</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A66" s="12" t="s">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A67" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="B66" s="12" t="s">
+      <c r="B67" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="C66" s="12"/>
-      <c r="D66" s="12"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A67" s="13" t="s">
+      <c r="C67" s="12"/>
+      <c r="D67" s="12"/>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A68" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="B67" s="14" t="s">
+      <c r="B68" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="C67" s="15" t="s">
+      <c r="C68" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D67" s="16" t="n">
+      <c r="D68" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K235</f>
         <v>237.936</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A68" s="13" t="s">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A69" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="B68" s="14" t="s">
+      <c r="B69" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="C68" s="15" t="s">
+      <c r="C69" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D68" s="16" t="n">
+      <c r="D69" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K246</f>
         <v>0.522275</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A69" s="12" t="s">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A70" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="B69" s="12" t="s">
+      <c r="B70" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C69" s="12"/>
-      <c r="D69" s="12"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A70" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="B70" s="19" t="s">
-        <v>121</v>
-      </c>
-      <c r="C70" s="15"/>
-      <c r="D70" s="16"/>
+      <c r="C70" s="12"/>
+      <c r="D70" s="12"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="B71" s="19" t="s">
+        <v>121</v>
+      </c>
+      <c r="C71" s="15"/>
+      <c r="D71" s="16"/>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A72" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="B71" s="14" t="s">
+      <c r="B72" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="C71" s="15" t="s">
+      <c r="C72" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D71" s="16" t="n">
+      <c r="D72" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K250</f>
         <v>65.5598924</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A72" s="13" t="s">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A73" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="B72" s="14" t="s">
+      <c r="B73" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="C72" s="15" t="s">
+      <c r="C73" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D72" s="16" t="n">
+      <c r="D73" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K282</f>
         <v>490.721915</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A73" s="13" t="s">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A74" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="B73" s="14" t="s">
+      <c r="B74" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="C73" s="15" t="s">
+      <c r="C74" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D73" s="16" t="n">
+      <c r="D74" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K293</f>
         <v>4140.49335597927</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A74" s="13" t="s">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A75" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="B74" s="14" t="s">
+      <c r="B75" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="C74" s="15" t="s">
+      <c r="C75" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D74" s="16" t="n">
+      <c r="D75" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K295</f>
         <v>919.697915</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A75" s="13" t="s">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A76" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="B75" s="14" t="s">
+      <c r="B76" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="C75" s="15" t="s">
+      <c r="C76" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D75" s="16" t="n">
+      <c r="D76" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K305</f>
         <v>128.904</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A76" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="B76" s="19" t="s">
-        <v>133</v>
-      </c>
-      <c r="C76" s="15"/>
-      <c r="D76" s="16"/>
-    </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B77" s="19" t="s">
+        <v>133</v>
+      </c>
+      <c r="C77" s="15"/>
+      <c r="D77" s="16"/>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A78" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="B77" s="14" t="s">
+      <c r="B78" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="C77" s="15" t="s">
+      <c r="C78" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="D77" s="16" t="n">
+      <c r="D78" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K309</f>
         <v>0.4125</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A78" s="13" t="s">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A79" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="B78" s="14" t="s">
+      <c r="B79" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="C78" s="15" t="s">
+      <c r="C79" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D78" s="16" t="n">
+      <c r="D79" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K312</f>
         <v>4.095</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A79" s="13" t="s">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A80" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B79" s="14" t="s">
+      <c r="B80" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="C79" s="15" t="s">
+      <c r="C80" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D79" s="16" t="n">
+      <c r="D80" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K316</f>
         <v>18.2336</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A80" s="13" t="s">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A81" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="B80" s="14" t="s">
+      <c r="B81" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="C80" s="15" t="s">
+      <c r="C81" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="D80" s="16" t="n">
+      <c r="D81" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K318</f>
         <v>1.5607</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A81" s="12" t="s">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A82" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="B81" s="12" t="s">
+      <c r="B82" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="C81" s="12"/>
-      <c r="D81" s="12"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A82" s="13" t="s">
+      <c r="C82" s="12"/>
+      <c r="D82" s="12"/>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A83" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="B82" s="14" t="s">
+      <c r="B83" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="C82" s="15" t="s">
+      <c r="C83" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="D82" s="16" t="n">
+      <c r="D83" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K321</f>
         <v>15.0</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A83" s="13" t="s">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A84" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="B83" s="14" t="s">
+      <c r="B84" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C83" s="15" t="s">
+      <c r="C84" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="D83" s="16" t="n">
+      <c r="D84" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K323</f>
         <v>162.69</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A84" s="13" t="s">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A85" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="B84" s="14" t="s">
+      <c r="B85" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="C84" s="15" t="s">
+      <c r="C85" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="D84" s="16" t="n">
+      <c r="D85" s="16" t="n">
         <f>+'PLANILLA GENERAL DE METRADOS'!K325</f>
         <v>78.42</v>
       </c>

</xml_diff>